<commit_message>
Login Testfälle + ausgewertet
</commit_message>
<xml_diff>
--- a/Testdaten/Testdaten von und für GPT-4/OpenCart-TestExecution Results_GPT-4_ausgewertet.xlsx
+++ b/Testdaten/Testdaten von und für GPT-4/OpenCart-TestExecution Results_GPT-4_ausgewertet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marvi\Desktop\Bachelor-Thesis\Testdaten\Testdaten von und für GPT-4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A7137E4-447F-46AB-AC64-74804BC924C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{565E8ED6-7CDE-4FDF-BEED-CDA4F0DF3832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Scenarios" sheetId="1" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="229">
   <si>
     <t>Test Scenario Description</t>
   </si>
@@ -209,14 +209,6 @@
   </si>
   <si>
     <t>Ja</t>
-  </si>
-  <si>
-    <t>TP = 1
-FP = 0
-TN = 0
-P = 1
-R = 1
-F1 = 1</t>
   </si>
   <si>
     <t>TC002</t>
@@ -235,15 +227,6 @@
     <t>All fields and Captcha should be visible</t>
   </si>
   <si>
-    <t>TP = 1
-FP = 0
-TN = 1
-Button "Register" wird nicht gecheckt
-P = 0,5
-R = 0,5
-F1 = 0,5</t>
-  </si>
-  <si>
     <t>TC003</t>
   </si>
   <si>
@@ -258,14 +241,6 @@
   </si>
   <si>
     <t>Error messages for all required fields</t>
-  </si>
-  <si>
-    <t>TP = 2
-FP = 0
-TN = 0
-P = 1
-R = 1
-F1 = 1</t>
   </si>
   <si>
     <t>TC004</t>
@@ -287,14 +262,6 @@
     <t>Welcome message appears, verification email is sent</t>
   </si>
   <si>
-    <t>TP = 5
-FP = 0
-TN = 0
-P = 1
-R = 1
-F1 = 1</t>
-  </si>
-  <si>
     <t>TC005</t>
   </si>
   <si>
@@ -312,14 +279,6 @@
     <t>Error: 'Username is already registered'</t>
   </si>
   <si>
-    <t>TP = 3
-FP = 0
-TN = 0
-P = 1
-R = 1
-F1 = 1</t>
-  </si>
-  <si>
     <t>TC006</t>
   </si>
   <si>
@@ -352,14 +311,6 @@
   </si>
   <si>
     <t>Error message for the missing field</t>
-  </si>
-  <si>
-    <t>TP = 2
-FP = 0
-TN = 1 Es wird nicht nach First Name und Last Name gecheckt
-P = 2/3
-R = 2/3
-F1 = 2/3</t>
   </si>
   <si>
     <t>TC008</t>
@@ -552,14 +503,6 @@
     <t>Entered details should persist (if implemented)</t>
   </si>
   <si>
-    <t>TP = 4
-FP = 0
-TN = 0
-P = 1
-R = 1
-F1 = 1</t>
-  </si>
-  <si>
     <t>TC019</t>
   </si>
   <si>
@@ -602,14 +545,6 @@
   <si>
     <t>(17/27) * 100
 = 62,9%</t>
-  </si>
-  <si>
-    <t>TP = 1
-FP = 0
-TN = 1, Es wird nicht geschaut ob auch "Opencart angezeigt wird", dies ist jedoch auch in der Leiste
-P = 0,5
-R = 0,5
-F1 = 0,5</t>
   </si>
   <si>
     <t>Open Login Page</t>
@@ -858,6 +793,110 @@
   </si>
   <si>
     <t>Login' button should be disabled (if implemented)</t>
+  </si>
+  <si>
+    <t>TP = 1
+FP = 0
+FN = 0
+P = 1
+R = 1
+F1 = 1</t>
+  </si>
+  <si>
+    <t>TP = 1
+FP = 0
+FN = 1
+Button "Register" wird nicht gecheckt
+P = 1
+R = 0,5
+F1 = 0,5</t>
+  </si>
+  <si>
+    <t>TP = 2
+FP = 0
+FN = 0
+P = 1
+R = 1
+F1 = 1</t>
+  </si>
+  <si>
+    <t>TP = 5
+FP = 0
+FN = 0
+P = 1
+R = 1
+F1 = 1</t>
+  </si>
+  <si>
+    <t>TP = 3
+FP = 0
+FN = 0
+P = 1
+R = 1
+F1 = 1</t>
+  </si>
+  <si>
+    <t>TP = 2
+FP = 0
+FN = 1 Es wird nicht nach First Name und Last Name gecheckt
+P = 2/3
+R = 2/3
+F1 = 2/3</t>
+  </si>
+  <si>
+    <t>TP = 4
+FP = 0
+FN = 0
+P = 1
+R = 1
+F1 = 1</t>
+  </si>
+  <si>
+    <t>TP = 1
+FP = 0
+FN = 1, Es wird nicht geschaut ob auch "Opencart angezeigt wird", dies ist jedoch auch in der Leiste
+P = 0,5
+R = 0,5
+F1 = 0,5</t>
+  </si>
+  <si>
+    <t>Falsches Erwartetes Ergebnis, die Funktion wurde nicht implementiert und GPT-4 wusste nicht ob es implementiert ist oder nicht</t>
+  </si>
+  <si>
+    <t>TP = 1
+FP = 0
+FN = 1
+Button "Register" wird nicht gecheckt
+P = 1
+R = 0,5
+F1 = 0,66</t>
+  </si>
+  <si>
+    <t>TP = 1
+FP = 0
+FN = 1, Es wird nicht geschaut ob auch "Opencart angezeigt wird", dies ist jedoch auch in der Leiste
+P = 1
+R = 0,5
+F1 = 0,66</t>
+  </si>
+  <si>
+    <t>TP = 2
+FP = 1, Es sind nur Punkte 
+FN = 0
+P = 2/3
+R = 1
+F1 = 0,8</t>
+  </si>
+  <si>
+    <t>TP = 2
+FP = 0
+FN = 1 Es wird nicht nach First Name und Last Name gecheckt
+P = 1
+R = 2/3
+F1 = 0,8</t>
+  </si>
+  <si>
+    <t>Anzahl positive Testfälle</t>
   </si>
 </sst>
 </file>
@@ -962,7 +1001,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1000,11 +1039,8 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1324,6 +1360,9 @@
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="B3">
+        <v>22</v>
+      </c>
     </row>
     <row r="4" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -1636,7 +1675,7 @@
         <v>47</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>48</v>
+        <v>215</v>
       </c>
       <c r="I2" s="9">
         <v>1</v>
@@ -1644,28 +1683,28 @@
     </row>
     <row r="3" spans="1:9" ht="135" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="C3" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" s="8" t="s">
+      <c r="E3" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="F3" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="F3" s="8" t="s">
-        <v>53</v>
-      </c>
       <c r="G3" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>54</v>
+        <v>224</v>
       </c>
       <c r="I3" s="12">
         <v>0</v>
@@ -1673,28 +1712,28 @@
     </row>
     <row r="4" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="E4" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C4" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D4" s="8" t="s">
+      <c r="F4" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="E4" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>59</v>
-      </c>
       <c r="G4" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>60</v>
+        <v>217</v>
       </c>
       <c r="I4" s="9">
         <v>1</v>
@@ -1702,28 +1741,28 @@
     </row>
     <row r="5" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="F5" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>65</v>
-      </c>
       <c r="G5" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>66</v>
+        <v>218</v>
       </c>
       <c r="I5" s="9">
         <v>1</v>
@@ -1731,28 +1770,28 @@
     </row>
     <row r="6" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>71</v>
-      </c>
       <c r="G6" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>72</v>
+        <v>219</v>
       </c>
       <c r="I6" s="9">
         <v>1</v>
@@ -1760,28 +1799,28 @@
     </row>
     <row r="7" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>72</v>
+        <v>219</v>
       </c>
       <c r="I7" s="9">
         <v>1</v>
@@ -1789,28 +1828,28 @@
     </row>
     <row r="8" spans="1:9" ht="135" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="G8" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>83</v>
+        <v>227</v>
       </c>
       <c r="I8" s="12">
         <v>0</v>
@@ -1818,28 +1857,28 @@
     </row>
     <row r="9" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="G9" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>72</v>
+        <v>219</v>
       </c>
       <c r="I9" s="9">
         <v>1</v>
@@ -1847,28 +1886,28 @@
     </row>
     <row r="10" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="G10" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>72</v>
+        <v>219</v>
       </c>
       <c r="I10" s="9">
         <v>1</v>
@@ -1876,28 +1915,28 @@
     </row>
     <row r="11" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="G11" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>72</v>
+        <v>219</v>
       </c>
       <c r="I11" s="9">
         <v>1</v>
@@ -1905,28 +1944,28 @@
     </row>
     <row r="12" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="G12" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>72</v>
+        <v>219</v>
       </c>
       <c r="I12" s="9">
         <v>1</v>
@@ -1934,28 +1973,28 @@
     </row>
     <row r="13" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="G13" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>72</v>
+        <v>219</v>
       </c>
       <c r="I13" s="9">
         <v>1</v>
@@ -1963,28 +2002,28 @@
     </row>
     <row r="14" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="G14" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>72</v>
+        <v>219</v>
       </c>
       <c r="I14" s="9">
         <v>1</v>
@@ -1992,28 +2031,28 @@
     </row>
     <row r="15" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="G15" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>72</v>
+        <v>219</v>
       </c>
       <c r="I15" s="9">
         <v>1</v>
@@ -2021,28 +2060,28 @@
     </row>
     <row r="16" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="G16" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>72</v>
+        <v>219</v>
       </c>
       <c r="I16" s="9">
         <v>1</v>
@@ -2050,28 +2089,28 @@
     </row>
     <row r="17" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="C17" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="G17" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>66</v>
+        <v>218</v>
       </c>
       <c r="I17" s="9">
         <v>1</v>
@@ -2079,28 +2118,28 @@
     </row>
     <row r="18" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="C18" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G18" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>72</v>
+        <v>219</v>
       </c>
       <c r="I18" s="9">
         <v>1</v>
@@ -2108,28 +2147,28 @@
     </row>
     <row r="19" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="C19" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="G19" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>139</v>
+        <v>221</v>
       </c>
       <c r="I19" s="9">
         <v>1</v>
@@ -2137,28 +2176,28 @@
     </row>
     <row r="20" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="G20" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>72</v>
+        <v>219</v>
       </c>
       <c r="I20" s="9">
         <v>1</v>
@@ -2166,34 +2205,37 @@
     </row>
     <row r="21" spans="1:9" ht="195" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="C21" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="G21" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H21" s="12" t="s">
-        <v>153</v>
+        <v>225</v>
       </c>
       <c r="I21" s="12">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="H22" s="11" t="s">
+        <v>228</v>
+      </c>
       <c r="I22" s="10">
         <f>SUM(I2:I21)</f>
         <v>17</v>
@@ -2201,7 +2243,7 @@
     </row>
     <row r="23" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="H23" s="11" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="I23" s="8">
         <v>27</v>
@@ -2209,10 +2251,10 @@
     </row>
     <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="H24" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -2312,7 +2354,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2118811-6422-40EF-BD37-945B8642CF7D}">
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" customWidth="1"/>
@@ -2321,536 +2363,702 @@
     <col min="4" max="4" width="22.42578125" customWidth="1"/>
     <col min="5" max="5" width="24.28515625" customWidth="1"/>
     <col min="6" max="6" width="22.28515625" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" customWidth="1"/>
+    <col min="8" max="8" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="G1" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="I2" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="I3" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="E4" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E2" s="11" t="s">
+      <c r="F4" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="G4" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="I4" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-    </row>
-    <row r="3" spans="1:9" ht="90" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="11" t="s">
+      <c r="C5" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="C3" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" s="11" t="s">
+      <c r="E5" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F5" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-    </row>
-    <row r="4" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="B4" s="11" t="s">
+      <c r="G5" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="I5" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="C4" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D4" s="11" t="s">
+      <c r="C6" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="E6" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="F6" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="I6" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="C7" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="E7" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-    </row>
-    <row r="5" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" s="11" t="s">
+      <c r="F7" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="C5" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" s="11" t="s">
+      <c r="G7" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="I7" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="C8" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="E8" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F8" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="I8" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-    </row>
-    <row r="6" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" s="11" t="s">
+      <c r="C9" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="E9" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="C6" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="E6" s="11" t="s">
+      <c r="F9" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="I9" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="F6" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
-    </row>
-    <row r="7" spans="1:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="B7" s="11" t="s">
+      <c r="C10" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="C7" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="E7" s="11" t="s">
+      <c r="E10" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F10" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-    </row>
-    <row r="8" spans="1:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="B8" s="11" t="s">
+      <c r="G10" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="I10" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="C8" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="E8" s="11" t="s">
+      <c r="C11" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="F8" s="11" t="s">
-        <v>172</v>
-      </c>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="11"/>
-    </row>
-    <row r="9" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="B9" s="11" t="s">
+      <c r="E11" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="C9" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="E9" s="11" t="s">
+      <c r="F11" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="F9" s="11" t="s">
-        <v>172</v>
-      </c>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-    </row>
-    <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="B10" s="11" t="s">
+      <c r="G11" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="I11" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A12" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="C10" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" s="11" t="s">
+      <c r="C12" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="E12" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="F12" s="8" t="s">
         <v>179</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="G12" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="I12" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="11"/>
-    </row>
-    <row r="11" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="B11" s="11" t="s">
+      <c r="C13" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="E13" s="8" t="s">
         <v>181</v>
       </c>
-      <c r="C11" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" s="11" t="s">
+      <c r="F13" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="I13" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="C14" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="E14" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F14" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="I14" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-    </row>
-    <row r="12" spans="1:9" ht="90" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="B12" s="11" t="s">
+      <c r="C15" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="C12" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="E12" s="11" t="s">
+      <c r="E15" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="F15" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
-    </row>
-    <row r="13" spans="1:9" ht="90" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="B13" s="11" t="s">
+      <c r="G15" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="I15" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="C13" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="E13" s="11" t="s">
+      <c r="C16" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>189</v>
       </c>
-      <c r="F13" s="11" t="s">
-        <v>172</v>
-      </c>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-    </row>
-    <row r="14" spans="1:9" ht="90" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="B14" s="11" t="s">
+      <c r="E16" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="C14" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="E14" s="11" t="s">
+      <c r="F16" s="8" t="s">
         <v>191</v>
       </c>
-      <c r="F14" s="11" t="s">
-        <v>172</v>
-      </c>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-    </row>
-    <row r="15" spans="1:9" ht="90" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="B15" s="11" t="s">
+      <c r="G16" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="I16" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="C15" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D15" s="11" t="s">
+      <c r="C17" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E17" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F17" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-    </row>
-    <row r="16" spans="1:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="B16" s="11" t="s">
+      <c r="G17" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="I17" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>196</v>
       </c>
-      <c r="C16" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D16" s="11" t="s">
+      <c r="C18" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="E18" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="F18" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>225</v>
+      </c>
+      <c r="I18" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="C19" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="E19" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-    </row>
-    <row r="17" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="B17" s="11" t="s">
+      <c r="F19" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="I19" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>200</v>
       </c>
-      <c r="C17" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D17" s="11" t="s">
+      <c r="C20" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="E20" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="F20" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="I20" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A21" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>202</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="C21" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="E21" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-    </row>
-    <row r="18" spans="1:9" ht="90" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="B18" s="11" t="s">
+      <c r="F21" s="8" t="s">
         <v>204</v>
       </c>
-      <c r="C18" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>201</v>
-      </c>
-      <c r="E18" s="11" t="s">
+      <c r="G21" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="I21" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
         <v>205</v>
       </c>
-      <c r="F18" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
-    </row>
-    <row r="19" spans="1:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="A19" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="B19" s="11" t="s">
+      <c r="B22" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="C19" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>201</v>
-      </c>
-      <c r="E19" s="11" t="s">
+      <c r="C22" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D22" s="8" t="s">
         <v>207</v>
       </c>
-      <c r="F19" s="14" t="s">
-        <v>222</v>
-      </c>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-    </row>
-    <row r="20" spans="1:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="B20" s="11" t="s">
+      <c r="E22" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="C20" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>201</v>
-      </c>
-      <c r="E20" s="11" t="s">
+      <c r="F22" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="F20" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-    </row>
-    <row r="21" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A21" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="B21" s="11" t="s">
+      <c r="G22" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="I22" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A23" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="C21" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="E21" s="11" t="s">
+      <c r="B23" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="F21" s="11" t="s">
+      <c r="C23" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="E23" s="8" t="s">
         <v>212</v>
       </c>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-    </row>
-    <row r="22" spans="1:9" ht="90" x14ac:dyDescent="0.25">
-      <c r="A22" s="11" t="s">
+      <c r="F23" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="B22" s="11" t="s">
-        <v>214</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D22" s="11" t="s">
+      <c r="G23" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H23" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="E22" s="11" t="s">
-        <v>216</v>
-      </c>
-      <c r="F22" s="11" t="s">
-        <v>217</v>
-      </c>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-    </row>
-    <row r="23" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A23" s="11" t="s">
-        <v>218</v>
-      </c>
-      <c r="B23" s="11" t="s">
-        <v>219</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>215</v>
-      </c>
-      <c r="E23" s="11" t="s">
-        <v>220</v>
-      </c>
-      <c r="F23" s="11" t="s">
-        <v>221</v>
-      </c>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
+      <c r="I23" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="G24" s="11"/>
+      <c r="H24" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="I24" s="8">
+        <f>SUM(I2:I23)</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="G25" s="11"/>
+      <c r="H25" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="I25" s="8">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G26" s="11"/>
+      <c r="H26" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="I26" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>